<commit_message>
Add LIFEBLOOM IP project, fix broken image refs, add media save protection
</commit_message>
<xml_diff>
--- a/项目索引.xlsx
+++ b/项目索引.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\.qoderworkcn\workspace\mqqksxuu2hjp0h49\outputs\portfolio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2954BF8C-ECF2-4D90-880E-F4DE35D8BF24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AA04012-490F-4CF8-AEDB-B2642E495952}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="101">
   <si>
     <t xml:space="preserve">一级分类 </t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -417,6 +417,18 @@
   </si>
   <si>
     <t>品牌定位 → 视觉策略 → 概念草图 → 色彩渲染 → 最终输出</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LIFEBLOOM</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>IP概念定义 → 形象线稿  → Logo设计→ 3D效果图 → 周边设计 → 品牌应用</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>一个以花朵拟人为核心视觉隐喻的时尚少女IP。以花朵为人格隐喻，创造一群拥有不同肤色、个性与时尚风格的年轻女孩。从Logo设计到立体效果图，完成原创IP的全案设计。包含IP形象设计、品牌标识、品牌配色、品牌应用等案例。</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1059,13 +1071,13 @@
     <xdr:from>
       <xdr:col>7</xdr:col>
       <xdr:colOff>217714</xdr:colOff>
-      <xdr:row>17</xdr:row>
+      <xdr:row>18</xdr:row>
       <xdr:rowOff>150634</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>2258785</xdr:colOff>
-      <xdr:row>17</xdr:row>
+      <xdr:row>18</xdr:row>
       <xdr:rowOff>2191705</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1109,13 +1121,13 @@
     <xdr:from>
       <xdr:col>7</xdr:col>
       <xdr:colOff>231321</xdr:colOff>
-      <xdr:row>18</xdr:row>
+      <xdr:row>19</xdr:row>
       <xdr:rowOff>301170</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>2122714</xdr:colOff>
-      <xdr:row>18</xdr:row>
+      <xdr:row>19</xdr:row>
       <xdr:rowOff>1562099</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1159,13 +1171,13 @@
     <xdr:from>
       <xdr:col>7</xdr:col>
       <xdr:colOff>299357</xdr:colOff>
-      <xdr:row>19</xdr:row>
+      <xdr:row>20</xdr:row>
       <xdr:rowOff>573350</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>2095500</xdr:colOff>
-      <xdr:row>19</xdr:row>
+      <xdr:row>20</xdr:row>
       <xdr:rowOff>1584032</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1209,13 +1221,13 @@
     <xdr:from>
       <xdr:col>7</xdr:col>
       <xdr:colOff>40822</xdr:colOff>
-      <xdr:row>20</xdr:row>
+      <xdr:row>21</xdr:row>
       <xdr:rowOff>503463</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>2305247</xdr:colOff>
-      <xdr:row>20</xdr:row>
+      <xdr:row>21</xdr:row>
       <xdr:rowOff>1639072</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1259,13 +1271,13 @@
     <xdr:from>
       <xdr:col>7</xdr:col>
       <xdr:colOff>95250</xdr:colOff>
-      <xdr:row>21</xdr:row>
+      <xdr:row>22</xdr:row>
       <xdr:rowOff>292526</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>2272393</xdr:colOff>
-      <xdr:row>21</xdr:row>
+      <xdr:row>22</xdr:row>
       <xdr:rowOff>1804127</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1309,13 +1321,13 @@
     <xdr:from>
       <xdr:col>7</xdr:col>
       <xdr:colOff>231322</xdr:colOff>
-      <xdr:row>23</xdr:row>
+      <xdr:row>24</xdr:row>
       <xdr:rowOff>272142</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>2143432</xdr:colOff>
-      <xdr:row>23</xdr:row>
+      <xdr:row>24</xdr:row>
       <xdr:rowOff>1351007</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1359,13 +1371,13 @@
     <xdr:from>
       <xdr:col>7</xdr:col>
       <xdr:colOff>149679</xdr:colOff>
-      <xdr:row>24</xdr:row>
+      <xdr:row>25</xdr:row>
       <xdr:rowOff>382185</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>2095500</xdr:colOff>
-      <xdr:row>24</xdr:row>
+      <xdr:row>25</xdr:row>
       <xdr:rowOff>1564070</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1409,13 +1421,13 @@
     <xdr:from>
       <xdr:col>7</xdr:col>
       <xdr:colOff>13607</xdr:colOff>
-      <xdr:row>25</xdr:row>
+      <xdr:row>26</xdr:row>
       <xdr:rowOff>622905</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
       <xdr:colOff>13607</xdr:colOff>
-      <xdr:row>25</xdr:row>
+      <xdr:row>26</xdr:row>
       <xdr:rowOff>1288143</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1459,13 +1471,13 @@
     <xdr:from>
       <xdr:col>7</xdr:col>
       <xdr:colOff>299358</xdr:colOff>
-      <xdr:row>26</xdr:row>
+      <xdr:row>27</xdr:row>
       <xdr:rowOff>27214</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>1993899</xdr:colOff>
-      <xdr:row>26</xdr:row>
+      <xdr:row>27</xdr:row>
       <xdr:rowOff>1298120</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1509,13 +1521,13 @@
     <xdr:from>
       <xdr:col>7</xdr:col>
       <xdr:colOff>68036</xdr:colOff>
-      <xdr:row>15</xdr:row>
+      <xdr:row>16</xdr:row>
       <xdr:rowOff>367392</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>2288722</xdr:colOff>
-      <xdr:row>15</xdr:row>
+      <xdr:row>16</xdr:row>
       <xdr:rowOff>1477735</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1547,6 +1559,56 @@
         <a:xfrm>
           <a:off x="18995572" y="26220963"/>
           <a:ext cx="2220686" cy="1110343"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>347382</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>77566</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>2072775</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>1804148</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="图片 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{80BB6C7B-1216-4E6F-ACC7-48541D218039}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId22" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="19240500" y="25996772"/>
+          <a:ext cx="1725393" cy="1726582"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1821,7 +1883,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:H29"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="31.375" style="1" customWidth="1"/>
@@ -2177,31 +2239,30 @@
         <v>76</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="137.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:8" ht="146.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>31</v>
+        <v>98</v>
       </c>
       <c r="D16" s="1">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="E16" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="F16" s="5" t="s">
-        <v>77</v>
+      <c r="F16" s="3" t="s">
+        <v>100</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="H16" s="1"/>
-    </row>
-    <row r="17" spans="1:8" ht="180" customHeight="1" x14ac:dyDescent="0.2">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="137.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
         <v>9</v>
       </c>
@@ -2209,25 +2270,23 @@
         <v>28</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="D17" s="1">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="E17" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="F17" s="3" t="s">
-        <v>33</v>
+      <c r="F17" s="5" t="s">
+        <v>77</v>
       </c>
       <c r="G17" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="H17" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" ht="181.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="H17" s="1"/>
+    </row>
+    <row r="18" spans="1:8" ht="180" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
         <v>9</v>
       </c>
@@ -2235,45 +2294,48 @@
         <v>28</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D18" s="1">
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="E18" s="1" t="s">
         <v>47</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="G18" s="3" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="19" spans="1:8" ht="149.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="H18" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" ht="181.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
         <v>9</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D19" s="1">
         <v>2022</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>79</v>
+        <v>36</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" ht="177.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" ht="149.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
         <v>9</v>
       </c>
@@ -2281,7 +2343,7 @@
         <v>29</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D20" s="1">
         <v>2022</v>
@@ -2290,13 +2352,13 @@
         <v>51</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" ht="164.25" customHeight="1" x14ac:dyDescent="0.2">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" ht="177.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
         <v>9</v>
       </c>
@@ -2304,53 +2366,53 @@
         <v>29</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D21" s="1">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" ht="174" customHeight="1" x14ac:dyDescent="0.2">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" ht="164.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
         <v>9</v>
       </c>
       <c r="B22" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D22" s="1">
+        <v>2023</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="F22" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="G22" s="3" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" ht="174" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B23" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="C22" s="1" t="s">
+      <c r="C23" s="1" t="s">
         <v>42</v>
-      </c>
-      <c r="D22" s="1">
-        <v>2025</v>
-      </c>
-      <c r="E22" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="F22" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="G22" s="3" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" ht="134.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>17</v>
       </c>
       <c r="D23" s="1">
         <v>2025</v>
@@ -2358,22 +2420,19 @@
       <c r="E23" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="F23" s="3" t="s">
-        <v>85</v>
+      <c r="F23" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="H23" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" ht="129.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" ht="134.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C24" s="1" t="s">
         <v>17</v>
@@ -2385,18 +2444,21 @@
         <v>47</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>96</v>
+        <v>85</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" ht="147.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>86</v>
+      </c>
+      <c r="H24" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" ht="129.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>92</v>
+        <v>44</v>
       </c>
       <c r="C25" s="1" t="s">
         <v>17</v>
@@ -2405,21 +2467,21 @@
         <v>2025</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" ht="144.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" ht="147.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C26" s="1" t="s">
         <v>17</v>
@@ -2431,18 +2493,18 @@
         <v>51</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="G26" s="3" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" ht="105" customHeight="1" x14ac:dyDescent="0.2">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" ht="144.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="C27" s="1" t="s">
         <v>17</v>
@@ -2451,16 +2513,39 @@
         <v>2025</v>
       </c>
       <c r="E27" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="F27" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="G27" s="3" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" ht="105" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D28" s="1">
+        <v>2025</v>
+      </c>
+      <c r="E28" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="F27" s="3" t="s">
+      <c r="F28" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="G27" s="1" t="s">
+      <c r="G28" s="1" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="29" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>